<commit_message>
fix excel function import duplication bug
</commit_message>
<xml_diff>
--- a/Excel/10_SolidWaste_WIP_v02.prename.bak.xlsx
+++ b/Excel/10_SolidWaste_WIP_v02.prename.bak.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA9B112-C757-4964-B4E2-8524ADAA9D82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C661AEBE-5F32-4721-A222-B9A323BAECFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Input - Solid waste" sheetId="70" r:id="rId4"/>
     <sheet name="10.1.1-2 Solid waste treatment" sheetId="69" r:id="rId5"/>
     <sheet name="Constants - Solid Waste" sheetId="110" r:id="rId6"/>
-    <sheet name="Constants - Common" sheetId="123" r:id="rId7"/>
+    <sheet name="Constants - Common" sheetId="124" r:id="rId7"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId8"/>
@@ -39,7 +39,17 @@
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Title">_xlfn.LAMBDA("Convert nitrous oxide emissions to carbon dioxide equivalent emissions")</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Unit">_xlfn.LAMBDA("t CO2e")</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Variable">_xlfn.LAMBDA("EN2O CO2e")</definedName>
-    <definedName name="Common_InputFunctions.Common_GetMCFTemperatureZone">_xlfn.LAMBDA(_xlpm.Temperature,_xlpm.MMS,_xlpm.TemperatureArray,_xlpm.MMSArray,_xlpm.ReturnArray, _xlfn.XLOOKUP(MEDIAN(_xlpm.Temperature, MIN(_xlpm.TemperatureArray), MAX(_xlpm.TemperatureArray)), _xlpm.TemperatureArray, _xlfn.XLOOKUP(_xlpm.MMS, _xlpm.MMSArray, _xlpm.ReturnArray)))</definedName>
+    <definedName name="Common_InputFunctions.Common_GetMCFTemperatureZone">_xlfn.LAMBDA(_xlpm.Temperature,_xlpm.MMS,_xlpm.TemperatureArray,_xlpm.MMSArray,_xlpm.ReturnArray,
+    _xlfn.XLOOKUP(
+        MEDIAN(
+            ROUND(_xlpm.Temperature, 0),
+            MIN(_xlpm.TemperatureArray),
+            MAX(_xlpm.TemperatureArray)
+        ),
+        _xlpm.TemperatureArray,
+        _xlfn.XLOOKUP(_xlpm.MMS, _xlpm.MMSArray, _xlpm.ReturnArray)
+    )
+)</definedName>
     <definedName name="Common_InputFunctions.CommonCropping_GetFracWET">_xlfn.LAMBDA(_xlpm.LeachingZone,_xlpm.ProductionSystem,_xlpm.LeachingZoneLookup,_xlpm.LeachingZoneFracWETLookup,_xlpm.ProductionSystemLookup,_xlpm.ProductionSystemFracWETLookup, _xlfn.LET(_xlpm.LeachingZoneFracWET, Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.LeachingZone, _xlpm.LeachingZoneLookup, _xlpm.LeachingZoneFracWETLookup), _xlpm.ProductionSystemFracWET, Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.ProductionSystem, _xlpm.ProductionSystemLookup, _xlpm.ProductionSystemFracWETLookup), IF(_xlpm.LeachingZoneFracWET + _xlpm.ProductionSystemFracWET &gt; 0, 1, 0)))</definedName>
     <definedName name="Common_InputFunctions.getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
     <definedName name="Common_InputFunctions.getOverlappingReportingPeriods">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), _xlpm.n, MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1), _xlpm.yrs, _xlfn.SEQUENCE(_xlpm.n, 1, _xlpm.firstYear, 1), _xlpm.starts, DATE(_xlpm.yrs, _xlpm.m, _xlpm.d), _xlpm.ends, _xlfn.MAP(_xlpm.starts, _xlpm.PeriodEnd), _xlpm.tag, IF(_xlpm.starts = _xlpm.ReportingCycleStart, " (This reporting cycle)", ""), _xlpm.startsText, TEXT(_xlpm.starts, "dd mmm yyyy"), _xlpm.endsText, TEXT(_xlpm.ends, "dd mmm yyyy"), IF(_xlpm.n = 0, "", _xlfn.HSTACK(_xlpm.startsText &amp; " to " &amp; _xlpm.endsText &amp; _xlpm.tag))))</definedName>
@@ -55,8 +65,17 @@
     <definedName name="Common_InputFunctions.Utility_LookupN2OEFFromProdIrrigationRainfall">_xlfn.LAMBDA(_xlpm.ProductionSystem,_xlpm.IrrigationMethod,_xlpm.RainfallZone,_xlpm.ProductionSystemArray,_xlpm.IrrigationMethodArray,_xlpm.RainfallZoneArray,_xlpm.ReturnArray, _xlfn.LET(_xlpm.IrrigationMethod, IF(_xlpm.IrrigationMethod = "Not irrigated", "Not irrigated", "Any"), _xlpm.RainfallZone, IF(_xlpm.IrrigationMethod = "Not irrigated", _xlpm.RainfallZone, "Any"), _xlfn.XLOOKUP(1, (_xlpm.ProductionSystemArray = _xlpm.ProductionSystem) * (_xlpm.IrrigationMethodArray = _xlpm.IrrigationMethod) * (_xlpm.RainfallZoneArray = _xlpm.RainfallZone), _xlpm.ReturnArray)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTable">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableNumber">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, IF(ISNUMBER(_xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, "")), _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""), 0))</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupValueInTableOneColumnAndHeader">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue1, _xlpm.LookupArray1, _xlfn.XLOOKUP(_xlpm.LookupValue2, _xlpm.LookupArray2, _xlpm.ReturnArray)))</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupValueInTableTwoColumns">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray, _xlfn.XLOOKUP(1, (_xlpm.LookupArray1 = _xlpm.LookupValue1) * (_xlpm.LookupArray2 = _xlpm.LookupValue2), _xlpm.ReturnArray, ""))</definedName>
+    <definedName name="Common_InputFunctions.Utility_LookupValueInTableOneColumnAndHeader">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray,_xlop.ValueIfFalse,
+    IFERROR(
+        _xlfn.XLOOKUP(_xlpm.LookupValue1, _xlpm.LookupArray1,
+            _xlfn.XLOOKUP(_xlpm.LookupValue2, _xlpm.LookupArray2, _xlpm.ReturnArray)
+        ),
+        IF(_xlfn.ISOMITTED(_xlpm.ValueIfFalse), "", _xlpm.ValueIfFalse)
+    )
+)</definedName>
+    <definedName name="Common_InputFunctions.Utility_LookupValueInTableTwoColumns">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray,_xlop.ValueIFFalse,
+    _xlfn.XLOOKUP(1, (_xlpm.LookupArray1=_xlpm.LookupValue1)*(_xlpm.LookupArray2=_xlpm.LookupValue2), _xlpm.ReturnArray, IF(_xlfn.ISOMITTED(_xlpm.ValueIFFalse), "", _xlpm.ValueIFFalse))
+)</definedName>
     <definedName name="Common_InputFunctions.Utility_ResultsItemFromEquationTitleAndSource">_xlfn.LAMBDA(_xlpm.TitleCell,_xlpm.SourceCell, SUBSTITUTE(LEFT(_xlpm.SourceCell, FIND(",", _xlpm.SourceCell) - 1), "VEERG 2026: ", "") &amp; " " &amp; _xlpm.TitleCell)</definedName>
     <definedName name="Common_InputFunctions.Utility_SourceHyperlink">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#'" &amp; _xlpm.sh &amp; "'!" &amp; _xlpm.addr))</definedName>
     <definedName name="Common_InputFunctions.Utility_SourceHyperlinkDifferentSheet">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#" &amp; _xlpm.addr))</definedName>
@@ -259,13 +278,21 @@
     <definedName name="WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume_Unit">_xlfn.LAMBDA("t")</definedName>
     <definedName name="WasteSolid_Equations.VEERG_10_1_1_1__2_MassOfWasteFromVolume_Variable">_xlfn.LAMBDA("Q_wt")</definedName>
     <definedName name="WasteSolid_InputFunctions.WasteSolid_InputFunctions_SumWasteTreatment">_xlfn.LAMBDA(_xlpm.TreatmentArray,_xlpm.WasteArray,_xlpm.TreatmentLocationArray,_xlpm.UnitArray,_xlpm.AmountArray,_xlpm.TreatmentType,_xlpm.WasteType,_xlpm.TreatmentLocationType,_xlpm.UnitType, SUMIFS(_xlpm.AmountArray, _xlpm.TreatmentArray, _xlpm.TreatmentType, _xlpm.WasteArray, _xlpm.WasteType, _xlpm.TreatmentLocationArray, _xlpm.TreatmentLocationType, _xlpm.UnitArray, _xlpm.UnitType))</definedName>
-    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(35, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Treatment type t","Waste type w","EFwt","EF source";"Landfill","Food waste (including animal carcasses, spoiled animal feed or crop)",2.1,"NGAF 2025 table 15";"Landfill","Paper and cardboard",3.3,"NGAF 2025 table 15";"Landfill","Green waste (including crop residues or prunings)",1.6,"NGAF 2025 table 15";"Landfill","Wood",0.7,"NGAF 2025 table 15";"Landfill","Textiles",2,"NGAF 2025 table 15";"Landfill","Sludge",0.4,"NGAF 2025 table 15";"Landfill","Rubber and leather",3.3,"NGAF 2025 table 15";"Landfill","Inert waste (including concrete, metal, plastic or glass)",0,"NGAF 2025 table 15";"Landfill","Municipal solid waste",1.6,"NGAF 2025 table 15";"Landfill","Commercial and industrial waste",1.3,"NGAF 2025 table 15";"Landfill","Construction and demolition waste",0.2,"NGAF 2025 table 15";"Incineration","Food waste, green waste, wood, sludge",0,"";"Incineration","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Incineration","Green waste (including crop residues or prunings)","","";"Incineration","Wood","","";"Incineration","Sludge","","";"Incineration","Paper and cardboard",0.0169,"";"Incineration","Textiles",0.3667,"";"Incineration","Rubber and leather",0.4919,"";"Incineration","Inert waste (including concrete, metal, plastic or glass)",0.11,"";"Incineration","Municipal solid waste",0.0537,"NGAF 2025 Table 18";"Incineration","Commercial and industrial waste",1.649,"NGAF 2025 Table 18";"Composting","All organic waste",0.046,"NGAF 2025 Table 19";"Composting","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Composting","Green waste (including crop residues or prunings)","","";"Composting","Wood","","";"Composting","Sludge","","";"Composting","Paper and cardboard","","";"Anaerobic digestion","All organic waste",0.028,"NGAF 2025 Table 19";"Anaerobic digestion","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Anaerobic digestion","Green waste (including crop residues or prunings)","","";"Anaerobic digestion","Wood","","";"Anaerobic digestion","Sludge","","";"Anaerobic digestion","Paper and cardboard","",""}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Data">_xlfn.LAMBDA(
+  _xlfn.MAKEARRAY(35, 4,
+    _xlfn.LAMBDA(_xlpm.r,_xlpm.c,
+      INDEX({"Treatment type t","Waste type w","EFwt","EF source";"Landfill","Food waste (including animal carcasses, spoiled animal feed or crop)",2.1,"NGAF 2025 table 15";"Landfill","Paper and cardboard",3.3,"NGAF 2025 table 15";"Landfill","Green waste (including crop residues or prunings)",1.6,"NGAF 2025 table 15";"Landfill","Wood",0.7,"NGAF 2025 table 15";"Landfill","Textiles",2,"NGAF 2025 table 15";"Landfill","Sludge",0.4,"NGAF 2025 table 15";"Landfill","Rubber and leather",3.3,"NGAF 2025 table 15";"Landfill","Inert waste (including concrete, metal, plastic or glass)",0,"NGAF 2025 table 15";"Landfill","Municipal solid waste",1.6,"NGAF 2025 table 15";"Landfill","Commercial and industrial waste",1.3,"NGAF 2025 table 15";"Landfill","Construction and demolition waste",0.2,"NGAF 2025 table 15";"Incineration","Food waste, green waste, wood, sludge",0,"";"Incineration","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Incineration","Green waste (including crop residues or prunings)","","";"Incineration","Wood","","";"Incineration","Sludge","","";"Incineration","Paper and cardboard",0.0169,"";"Incineration","Textiles",0.3667,"";"Incineration","Rubber and leather",0.4919,"";"Incineration","Inert waste (including concrete, metal, plastic or glass)",0.11,"";"Incineration","Municipal solid waste",0.0537,"NGAF 2025 Table 18";"Incineration","Commercial and industrial waste",1.649,"NGAF 2025 Table 18";"Composting","All organic waste",0.046,"NGAF 2025 Table 19";"Composting","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Composting","Green waste (including crop residues or prunings)","","";"Composting","Wood","","";"Composting","Sludge","","";"Composting","Paper and cardboard","","";"Anaerobic digestion","All organic waste",0.028,"NGAF 2025 Table 19";"Anaerobic digestion","Food waste (including animal carcasses, spoiled animal feed or crop)","","";"Anaerobic digestion","Green waste (including crop residues or prunings)","","";"Anaerobic digestion","Wood","","";"Anaerobic digestion","Sludge","","";"Anaerobic digestion","Paper and cardboard","",""}, _xlpm.r, _xlpm.c)
+)))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Source">_xlfn.LAMBDA(("VEERG 2026: Table A.4.1.1"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Title">_xlfn.LAMBDA(("Emission factors for wastes disposed of at different treatment facilities"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Unit">_xlfn.LAMBDA(("t CO2e / t"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variable">_xlfn.LAMBDA(("EFwt"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_EmissionFactorsForWasteTreatment_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(7, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION ON SOURCE:";"Fixed typo 'paper and carboard' to 'paper and cardboard'";"Fixed typo 'prunnings' to 'prunings'";"Added EF source column with specific references";"Added sub-categories for 'Incineration: Food waste, green waste, wood, sludge' in order to use volume to mass conversion factor values";"Added sub-categories for 'Composting: All organic waste' in order to use volume to mass conversion factor values";"Added sub-categories for 'Anaerobic digestion: All organic waste' in order to use volume to mass conversion factor values"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(12, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Waste type w","VTMw";"Food waste (including animal carcasses, spoiled animal feed or crop)",0.5;"Paper and cardboard",0.09;"Green waste (including crop residues or prunings)",0.24;"Wood",0.15;"Textiles",0.14;"Sludge",0.72;"Rubber and leather",0.14;"Inert waste (including concrete, metal, plastic or glass)",0.42;"Municipal solid waste",0.36;"Commercial and industrial waste",0.33;"Construction and demolition waste",0.39}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Data">_xlfn.LAMBDA(
+  _xlfn.MAKEARRAY(12, 2,
+    _xlfn.LAMBDA(_xlpm.r,_xlpm.c,
+      INDEX({"Waste type w","VTMw";"Food waste (including animal carcasses, spoiled animal feed or crop)",0.5;"Paper and cardboard",0.09;"Green waste (including crop residues or prunings)",0.24;"Wood",0.15;"Textiles",0.14;"Sludge",0.72;"Rubber and leather",0.14;"Inert waste (including concrete, metal, plastic or glass)",0.42;"Municipal solid waste",0.36;"Commercial and industrial waste",0.33;"Construction and demolition waste",0.39}, _xlpm.r, _xlpm.c)
+)))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Source">_xlfn.LAMBDA(("VEERG 2026: Table A.4.1.2"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Title">_xlfn.LAMBDA(("Volume to mass conversion factor for various waste types"))</definedName>
     <definedName name="WasteSolid_SourceData.Waste_WasteVolumeToMassConversion_Unit">_xlfn.LAMBDA(("t/m3"))</definedName>
@@ -4471,16 +4498,16 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{9FFE9889-DB7A-4270-AB8E-FB7F2B1CE390}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{4E11BF5D-46B6-4FC4-8EE1-5686DB1674D9}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{BB95A605-0301-47D2-8561-20055CE5D8B8}" name="Gas">
+    <tableColumn id="1" xr3:uid="{94ED37DE-10C8-4707-927B-378DA731DAB5}" name="Gas">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8EFA7C99-5555-4C4B-8F95-3D8FB2414AA7}" name="CO2-e factor">
+    <tableColumn id="2" xr3:uid="{DB1FD19B-CBF8-478A-85D5-0807B29F6E45}" name="CO2-e factor">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4489,7 +4516,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{8787881E-B5ED-4048-9E6C-432213D42BF6}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{9100ED4E-373D-484B-9A2F-5CE9A7918536}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4498,19 +4525,19 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{744726ED-B1FE-40EF-B079-F278265B77A9}" name="Gas">
+    <tableColumn id="1" xr3:uid="{340F5EBB-52DD-47F4-87F5-879EF314947C}" name="Gas">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{58D8E2CB-96B5-41C2-9627-1494ACE4BF3A}" name="Conversion factor">
+    <tableColumn id="5" xr3:uid="{4472DC72-BBC4-45A1-B318-351CF035E1D9}" name="Conversion factor">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8F158569-8E74-483C-A2DB-23C97B6DB59B}" name="Conversion factor 1">
+    <tableColumn id="2" xr3:uid="{86B3479F-B6E6-4B84-8B4E-87137929C5A7}" name="Conversion factor 1">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{415FBFBB-9E72-442F-BA60-974F40A04C83}" name="Conversion factor 2">
+    <tableColumn id="3" xr3:uid="{81EAB478-601A-4D01-9E3A-AFD0EB242430}" name="Conversion factor 2">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A2E33637-70DF-4FC1-B569-92546D025BCC}" name="Conversion factor combined">
+    <tableColumn id="4" xr3:uid="{68511CDC-DC5A-46AD-B652-010C2B145B20}" name="Conversion factor combined">
       <calculatedColumnFormula>Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 1]]/Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 2]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4519,7 +4546,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{E6C32F02-2B6E-4E9F-B607-2B8B63BB362A}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{4F338BC4-371F-40BB-B6D6-EDBEC5F35CA3}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4539,52 +4566,52 @@
     <filterColumn colId="15" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{B93BEB65-AF0E-4C90-A5E5-2D6C095B8E2D}" name="Climate zone" totalsRowCellStyle="Content bold">
+    <tableColumn id="1" xr3:uid="{67822301-B92A-4B61-A1C0-0ADC3942DD06}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E3049BCD-43E3-4DA5-9F9A-4E810AF004AE}" name="MAT" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{D110A3B8-D6C8-4CC4-BB4A-4D200FA18648}" name="MAT" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{6778AC6D-9EA3-4726-BB37-C4C302E023BE}" name="MAP" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{63D3AD49-7CAE-422D-8385-8F44E81D27A2}" name="MAP" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{9205BA52-00C0-4A68-BEC0-66085F975849}" name="Frost days per year" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{0E61174D-AFF3-49A8-9DD8-3395F9625C21}" name="Frost days per year" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{05E5E70C-20C9-464C-AE0D-13A2A3C6C2B8}" name="Elevation" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{778D3BC4-3182-446F-8AB1-E808355A50B0}" name="Elevation" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{D7170E68-B448-488C-90AF-84036666008E}" name="MAP:PET" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{1C576C14-C00A-45FA-8E44-66CABEF8A692}" name="MAP:PET" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{E83FE6F4-2A82-44C6-AA23-2FADCB8DC2C8}" name="Min temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{FD93130C-9DF4-4A7E-A4AF-449FED4E3936}" name="Min temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B5D23C21-D941-498A-9DB6-89B9400105B3}" name="Max temp" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{99EEFECB-D181-4B39-81A8-293D4B6B93C3}" name="Max temp" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{7F4E5732-0B15-442D-BBFB-60AC2FE76284}" name="Min rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{46AA20B4-99E8-4643-BEEC-1A29869133C5}" name="Min rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{9553CDCD-553F-440C-AE8A-05D24A44B78A}" name="Max rainfall" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{B2E26E39-F50D-4CAA-9CCB-217DAD608376}" name="Max rainfall" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{DC570CD3-2687-4CF1-99FB-A474CB114219}" name="Min frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{FEE83E36-C961-4C87-83A3-7F7DCF023ECE}" name="Min frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{EAD83885-16BD-4EB7-ACE0-D689AA0791CF}" name="Max frost days" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{2F3BD8C2-BF7B-43E5-BD35-330F80F727EC}" name="Max frost days" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{B1D062CB-88B9-473C-8630-40117CA5FCCA}" name="Min elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{E9FD1D3D-81D8-4260-A602-ED6CF28F529E}" name="Min elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{84C85017-70D3-4C86-B59A-01F1D4684039}" name="Max elevation" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{06800DC9-80FD-408B-AC00-AE0EE814199B}" name="Max elevation" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{527A0EA4-49A6-49A9-9D43-4D0A1F14E4F4}" name="Min MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{61F35B3A-50B3-45AB-8238-4701628F517C}" name="Min MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{ED08BACF-E556-472A-9C44-7E29C712AEAA}" name="Max MAP:PET" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{C1147147-2D1C-4CAC-B765-06AF6B72BF29}" name="Max MAP:PET" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4593,16 +4620,16 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{E7237802-B9F7-423C-B931-9690EC677252}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{8565CC95-7FE7-4070-9E4B-6173ADEAC3EF}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2F3C5BF6-EF08-4F1E-9F94-FBB9E2750D1E}" name="Climate zone" totalsRowCellStyle="Content bold">
+    <tableColumn id="1" xr3:uid="{FE8E81D7-E344-4DCA-9510-1F4F4940C680}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6FE57F93-CA38-4486-B5F4-31E7F3515273}" name="Wet or Dry Zone" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{C1DE0B72-F913-4F81-930B-BA174DD88102}" name="Wet or Dry Zone" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4611,7 +4638,7 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{0CEC90EE-94D5-4847-9C21-C52FACE64426}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{AD7A453A-960E-48C4-818E-88A5A4E9B232}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4619,16 +4646,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E39DA32C-1C64-4BA7-B875-E0A1E3EBA71D}" name="Temperature Zone">
+    <tableColumn id="1" xr3:uid="{30C665A5-58B3-4C9A-813D-6169BEA75E87}" name="Temperature Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{AA069C74-75BD-4B56-8FAE-E4509EE8157C}" name="MAT">
+    <tableColumn id="2" xr3:uid="{C4BD658F-8B2C-4E50-B9AA-768C61AD8D33}" name="MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3E25D1F7-6FE9-4B06-8074-EFC399DA617E}" name="Min MAT">
+    <tableColumn id="3" xr3:uid="{2B7351D1-6E8F-4339-9A61-8D1587C33530}" name="Min MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{0777ADDA-FF5A-4D7C-A562-45DB7D3E07CA}" name="Max MAT">
+    <tableColumn id="4" xr3:uid="{290957F6-BC5A-4EC9-BE34-463409E91886}" name="Max MAT">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4637,7 +4664,7 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{B22EBB8C-C001-420C-8E15-CE6791DDE453}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{71A46C27-7B40-4DAA-8A4E-FC2BD2A71782}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4645,16 +4672,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{07CB8351-7E0C-4F38-B8AB-A3C6EDA7FB09}" name="Rainfall Zone">
+    <tableColumn id="1" xr3:uid="{1295A534-1EFB-4C58-835D-7AD7327E4628}" name="Rainfall Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6C47BF53-6F7B-4971-A2FC-4986FBA21309}" name="Annual rainfall">
+    <tableColumn id="2" xr3:uid="{2C61115E-CDF3-4873-87E0-9805AF906A52}" name="Annual rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{23508B53-9533-4A71-999A-260EC2E71E72}" name="Min rainfall">
+    <tableColumn id="3" xr3:uid="{DD0441B2-DBBB-4ED5-AA3E-5F59C94C3F71}" name="Min rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{1FD44B6E-0A60-4BF6-87B8-0482E70DD058}" name="Max rainfall">
+    <tableColumn id="4" xr3:uid="{E49FDF78-F3E0-4418-A6B3-24FF34C6973B}" name="Max rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4663,16 +4690,16 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{8CFDCB87-3EC9-4565-801B-020F9EE627D4}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{598D7264-7AEC-46CF-BDD3-404DCC4F4819}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
   <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{6DE5CE44-BC58-44D3-8885-D73DE323EA8D}" name="Leaching Zone">
+    <tableColumn id="1" xr3:uid="{2A7B10A7-DC7B-43BB-B3E9-E15A56E10BF7}" name="Leaching Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{9E7A9332-E8E6-4EAA-96E9-14B4C43F0478}" name="Leaching criteria">
+    <tableColumn id="2" xr3:uid="{A029DFCF-4F57-4109-9755-386A00E5DFFF}" name="Leaching criteria">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4681,16 +4708,16 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{23D8D08B-46AB-4CD1-B9AA-ABBD27125754}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{933E20FC-D22D-4D59-919D-15188DD657E3}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
   <autoFilter ref="D153:E158" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{8BAAFFF3-40EE-4859-941F-2A3A0485D154}" name="Data source">
+    <tableColumn id="1" xr3:uid="{94667DCD-2ACB-42F8-AF02-5E5474B368B6}" name="Data source">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8D4AF151-0F61-40BF-B183-0FC77C6C936C}" name="Data score">
+    <tableColumn id="2" xr3:uid="{F91525D4-0D98-4E2D-BA84-0614DCA0CA0C}" name="Data score">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4699,16 +4726,16 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{197999FD-A2F5-46AB-A495-3324EE45AE16}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{4E67B181-9330-4F32-9F09-1980C61417E4}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DE39ECAC-1FB2-4195-8FE4-06DA3F94FFCF}" name="Is in leaching zone">
+    <tableColumn id="1" xr3:uid="{D7859584-A9EC-49C4-8B9A-7F33C0B13ECE}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DC31DA39-336E-49B9-84C4-3E076E605E08}" name="FracWET" dataDxfId="19">
+    <tableColumn id="2" xr3:uid="{99474450-C935-4FB3-AE11-97261C3096BB}" name="FracWET" dataDxfId="19">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4717,7 +4744,7 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{C46F92FD-2EF0-4BB4-9C10-10E9B7B93E2F}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{015DE67C-B31B-45F1-B56E-D1FE0F672A6F}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
   <autoFilter ref="D186:H199" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4726,19 +4753,19 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{B363E57D-D52F-41DC-8FA3-A71928F674E2}" name="Production system j">
+    <tableColumn id="1" xr3:uid="{9DB66CE7-3027-47A9-ABF1-872361D1DFA0}" name="Production system j">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3CBDD86-F1A1-476C-BFBE-68EA79BE93F7}" name="EFN2O">
+    <tableColumn id="2" xr3:uid="{D4D8B6E7-F7AC-40BD-BE81-FA553143E463}" name="EFN2O">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E5A75355-A9C5-4C57-876D-072AEB0934D4}" name="Production system only">
+    <tableColumn id="3" xr3:uid="{EA132FED-B045-4A84-93D7-38BA5A85F589}" name="Production system only">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A526F00A-A2CF-4C9A-9F14-871753E02424}" name="Irrigation method">
+    <tableColumn id="4" xr3:uid="{A7620288-1BD9-43A3-91A0-8E84DA84A7EE}" name="Irrigation method">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DBA8C250-FF6E-4158-A5E8-423BEC11735E}" name="Rainfall zone">
+    <tableColumn id="5" xr3:uid="{1D8830B5-FEA0-4AE5-A400-BCA0193D20BC}" name="Rainfall zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4773,16 +4800,16 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{D6985B42-7AC2-4929-93FA-D125EC2E237A}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="37" xr:uid="{2845EE53-0D5B-4F20-B1B2-3499AAE90F98}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{EACFD210-496F-4675-8157-B30417106278}" name="Irrigation type i">
+    <tableColumn id="1" xr3:uid="{CFA3EC27-6140-43DB-A4A8-23E72783F1A8}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F79672EE-4062-4666-B01F-CFAEB233AD5F}" name="FracWET" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{73D55980-D77E-4DC1-B406-1B61E6429787}" name="FracWET" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4791,16 +4818,16 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{92D61437-8BF3-4AFE-9BDA-FB7DCA9DF376}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="38" xr:uid="{45CD733D-0B1E-468A-9F20-FFCF95BABF61}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
   <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{49ACCBE6-0488-4580-80F9-8782996820E3}" name="Climate zone">
+    <tableColumn id="1" xr3:uid="{05E76E9A-E15A-4F9E-8E3D-EB4E6A878AD2}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2F36A480-8075-4EA6-90EE-3D16BA16A068}" name="EFPRP" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{F3D8D1B0-05E4-4393-A4DE-9E8B7F6AB615}" name="EFPRP" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4809,16 +4836,16 @@
 </file>
 
 <file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{C11F09FB-5C4C-4254-A5ED-9D42ABEE2161}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="39" xr:uid="{505BF33B-2B47-4AF9-820B-1263D6B51526}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
   <autoFilter ref="D212:E224" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{01ED90E4-3E1A-4247-B6D4-0819D55B9090}" name="Month">
+    <tableColumn id="1" xr3:uid="{AE4BBE37-76D1-4461-B191-9A5F56CBEBC4}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6088EA4E-6980-4526-A397-0F1E411826C8}" name="Season" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{570DC661-C85C-4579-AD94-4EF4C3DD1C88}" name="Season" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4827,7 +4854,7 @@
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{9CD4EEFF-6EDF-4839-89B8-2930EEF829B1}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="40" xr:uid="{10AAA4A6-AF97-4D1E-8472-CEF4CDB6ADC2}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
   <autoFilter ref="D231:S250" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4847,52 +4874,52 @@
     <filterColumn colId="15" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{59949994-8279-45A0-83D7-035F6BEFA7FA}" name="Temperature zone">
+    <tableColumn id="1" xr3:uid="{3974E62A-3C49-4285-89C8-37A7B89586D4}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1EFFE624-56DB-44BB-9BFA-561301531B47}" name="MAT (ºC)" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{FBF3C2C0-6AD3-4C8D-ABB0-E7B55A161A2D}" name="MAT (ºC)" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{37D82049-DA48-4A7B-B605-79F60792837A}" name="Anaerobic lagoon" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{4975F74F-EB9F-441D-9166-AAD936585BB8}" name="Anaerobic lagoon" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{72F9117F-D7D0-40B8-9EB0-61A02F8FD933}" name="Digester / covered lagoons" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{64812E07-9288-46A7-A401-AF11EDA3CFBA}" name="Digester / covered lagoons" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{37F2E3D9-133C-428F-A879-C1582770FE5B}" name="Liquid systems" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5465B090-6E3A-4C8A-AEEB-EB4C264FBA09}" name="Liquid systems" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8ED5D9EC-BECB-4243-9078-AAA6008F1F93}" name="Daily spread" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{864397B0-9134-4A49-BB40-FC9465A38B81}" name="Daily spread" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{EC4B3BCF-A8D1-4CA5-8842-82BA7EC27901}" name="Composting (passive windrow)" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{F42E6207-A033-49BC-A1ED-2E312F13F7D3}" name="Composting (passive windrow)" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D34377BD-6747-4FB1-A845-D7AE584F3DDF}" name="Solid storage" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{89788B0E-6AF3-4674-B148-58DB5B69F4D6}" name="Solid storage" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{8DCAB6F3-06C7-4FD8-AD49-A69C013377FA}" name="Pit storage" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{569A6AD9-6C2E-45E6-AF26-F1A8423DCACA}" name="Pit storage" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{7CCD1A15-23B9-43DD-A72B-8E1136E5B215}" name="Deep litter" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{4CAE90FD-F721-4A6C-9117-9960CC921BB4}" name="Deep litter" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{8E317F53-635D-4F0D-80FD-9E59AFFADA18}" name="Poultry manure with bedding" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{FDA78419-FAD8-4F70-8146-4333D6B2C100}" name="Poultry manure with bedding" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D05184FD-7DD0-487E-BA95-5C104A00EB9E}" name="Poultry manure without bedding" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{0EEC7F94-DE8A-41C5-9BCA-D9D16A0DD7E8}" name="Poultry manure without bedding" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{C695B47C-A416-4CEC-91A6-06805C0383C7}" name="Direct processing" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{C85C28A0-0713-4787-BD1D-84479B15C571}" name="Direct processing" dataDxfId="4" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{62B8BD67-F5E3-40C3-8665-D6706BF4340C}" name="Direct application" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{C016AE28-FDCB-409F-AE3E-76589E210CA5}" name="Direct application" dataDxfId="3" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{43A6140F-B453-4C23-8D30-B960C987223C}" name="Pasture range and paddock" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{A84AE0C5-5694-4C4B-A976-09D86C5DCE27}" name="Pasture range and paddock" dataDxfId="2" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{A2EE13F3-6006-4291-B949-2CE07450CD04}" name="MAT raw" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{9F8434F6-5AD8-48FE-9AA3-F852E841EF5F}" name="MAT raw" dataDxfId="1" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4901,16 +4928,16 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{91ED3876-12EB-4845-AA85-EA305D007C80}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="41" xr:uid="{EFD2F056-1354-4F51-AD8A-C51365131136}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
   <autoFilter ref="D257:E259" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{86C60C10-AF7E-4637-A69D-EB74DADDDD54}" name="Climate Zone">
+    <tableColumn id="1" xr3:uid="{25B37FDD-B4F6-411F-B208-73E52BB3F228}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EA9DCAE5-7F43-418E-9BA7-1DED83E2B0E1}" name="EFNi &amp; EFN2Oi" dataDxfId="0" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{EA53843A-9209-484C-BA92-4F5FC3B0749B}" name="EFNi &amp; EFN2Oi" dataDxfId="0" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4993,20 +5020,20 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{78C5FCE3-4615-4DB1-B2C1-5E2D0C5241EA}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E502FDA1-5AC3-46B4-B7EF-8C6C81E8F49F}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
   <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{36712EC9-CFBB-4111-90A4-6DBCD3A6C6BB}" name="State/Territory">
+    <tableColumn id="1" xr3:uid="{3456D280-C48E-4D73-9F38-6C177C5064C2}" name="State/Territory">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4EB4D251-45CF-4375-86D1-C01FF51BC565}" name="Common Name">
+    <tableColumn id="2" xr3:uid="{4C73AA57-72FC-4D0C-B42E-41D57F96A62F}" name="Common Name">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{2A36FDD0-8FF6-4303-9AB4-5D2982713930}" name="Abbreviation">
+    <tableColumn id="3" xr3:uid="{6E249920-6A25-4D2E-A9BF-A8AC2A072000}" name="Abbreviation">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5015,12 +5042,12 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{17558D75-72E8-4716-BF0C-E8CD2832237B}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C048262D-B831-408A-8F0D-67640401CC80}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
   <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B5DA7235-517D-42C4-8A1B-E7936561E620}" name="SA 4 Name">
+    <tableColumn id="1" xr3:uid="{4F266D0B-CED8-4355-A138-6E87957BA871}" name="SA 4 Name">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -12364,7 +12391,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1463CAFD-AACE-422D-94B8-8A91509A7C06}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D7999F-41BE-4BD1-A9FB-BA86B1408DF5}">
   <dimension ref="A1:BY259"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -16356,21 +16383,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxADoAIABXAGEAcwB0AGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AbABpAGQAIABXAGEAcwB0AGUAIABUAHIAZQBhAHQAbQBlAG4AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXABuAEUAXwBnAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAGcAPQBcAFwAcwB1AG0AXwB0AFwAXABzAHUAbQBfAHcAKABRAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB3AHQAZwApAFwAbgBRAF8AdwB0ACAAPQAgAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAIAAoAHQAKQBcAG4ARQBGAF8AdwB0AGcAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAdAAgAEMATwAyAGUALwB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AdwB0ACwAIABFAEYAXwB3AHQAZwAsAFwAbgAgACAAIAAgAFEAXwB3AHQAIAAqACAARQBGAF8AdwB0AGcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdABcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHcAKABRAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewB3AHQAZwB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzAFwAIgAsACAAXAAiAHQAXAAiACwAIABcACIAUwB1AG0AIABvAGYAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAHcAdABnAFwAIgAsACAAXAAiAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAdAAgAEMATwAyAGUALwB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGcAXAAiACwAIABcACIAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHYAbwBsAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAdgBvAGwAdQBtAGUAIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAdABvAG4AbgBlAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAxADAALgAxAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAG0AYQBzAHMAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AYQBzAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAIAB2AGEAcgBpAGEAYgBsAGUAcwAgAHQAbwAgAGMAbABlAGEAcgBsAHkAIAB0AHIAYQBjAGsAIABpAG4AcAB1AHQAIABvAHIAIABjAGEAbABjAHUAbABhAHQAZQBkACAAUQAgAHYAYQBsAHUAZQBzAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXABuAFEAXwB3AHQAXABuAHQAXABuAFEAXwB3AHQAPQBWAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXABuAFYAXwB3AHQAIAA9ACAAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAG0AMwApAFwAbgBWAFQATQBfAHcAIAA9ACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgACgAdAAvAG0AMwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAXwB3AHQALAAgAFYAVABNAF8AdwAsAFwAbgAgACAAIAAgAFYAXwB3AHQAIAAqACAAVgBUAE0AXwB3AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AdwB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB7AHcAdAB9AD0AVgBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBfAHcAdABcACIALAAgAFwAIgB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgBtADMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFQATQBfAHcAXAAiACwAIABcACIAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgB0AC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBGAHcAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAgAEMATwAyAGUAIAAvACAAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADEAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADUALAAgADQALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIAB0AHkAcABlACAAdABcACIALAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBFAEYAdwB0AFwAIgAsACAAXAAiAEUARgAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAyAC4AMQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMQA2ADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMwA2ADYANwAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADQAOQAxADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAXAB1ADAAMAAyADcAcABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBiAG8AYQByAGQAXAB1ADAAMAAyADcAIAB0AG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAdQAwADAAMgA3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAHIAdQBuAG4AaQBuAGcAcwBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAcgB1AG4AaQBuAGcAcwBcAHUAMAAwADIANwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABFAEYAIABzAG8AdQByAGMAZQAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAcABlAGMAaQBmAGkAYwAgAHIAZQBmAGUAcgBlAG4AYwBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgA6ACAARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQBcAHUAMAAwADIANwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBDAG8AbQBwAG8AcwB0AGkAbgBnADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAB1ADAAMAAyADcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAXAB1ADAAMAAyADcAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgA6ACAAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAdQAwADAAMgA3ACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAOgAgAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwAgACgAdAAvAG0AMwApACAAKABWAFQATQB3ACkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBUAE0AdwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgB0AC8AbQAzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADIALAAgADIALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAVgBUAE0AdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4ANQAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAuADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMQA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADcAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAuADQAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG4AcwB0AHIAdQBjAHQAaQBvAG4AIABhAG4AZAAgAGQAZQBtAG8AbABpAHQAaQBvAG4AIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA5AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBoAGEAbgBnAGUAZAAgAGMAbwBsAHUAbQBuACAAaABlAGEAZABlAHIAIABDAEYAdwAgAHQAbwAgAFYAVABNAHcAIAB0AG8AIABtAGEAdABjAGgAIAB0AGkAdABsAGUAIAB2AGEAcgBpAGEAYgBsAGUALgBcACIAKQApADsAXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsACAAVwBhAHMAdABlAFQAeQBwAGUALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABVAG4AaQB0AFQAeQBwAGUALABcAG4AIAAgAFMAVQBNAEkARgBTACgAXABuACAAIAAgACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAXABuACAAIAAgACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFwAbgAgACAAIAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABVAG4AaQB0AFQAeQBwAGUAXABuACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0ACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -16565,7 +16577,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -16574,26 +16586,22 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAZQBuAHQAZQByAHAAcgBpAHMAZQAgAHQAeQBwAGUAcwBcAG4ARQB4AGMAZQBsACAAbQBvAGQAdQBsAGUAIABuAGEAbQBlADoAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXABuAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAAoADAALgA2ADcAOAA0ACAAawBnAC8AbQAzACkAXABuAFQAYQBrAGUAbgAgAGYAcgBvAG0AIAB0AGgAZQAgAE4AYQB0AGkAbwBuAGEAbAAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABhAG4AZAAgAEUAbgBlAHIAZwB5ACAAUgBlAHAAbwByAHQAaQBuAGcAIABcAG4AKABNAGUAYQBzAHUAcgBlAG0AZQBuAHQAKQAgAEQAZQB0AGUAcgBtAGkAbgBhAHQAaQBvAG4AIAAyADAAMAA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHAAIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBtADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgAxAGEAXwAyACwAIAAzAC4AQgAuADEAYwBfADIALAAgADMALgBCAC4AMwBfADEALAAgADMALgBCAC4ANABnAF8AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADYANwA4ADQAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAFwAbgBDAGcAIAA9ACAANAA0AC8AMgA4ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAYQBjAHQAbwByAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANAA0AC8AMgA4ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAFwAbgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAZwBhAHMAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAAxAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAXAAiADQANAAvADEAMgBcACIALAAgADQANAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMASAA0AFwAIgAsACAAXAAiADEANgAvADEAMgBcACIALAAgADEANgAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AMgBPAFwAIgAsACAAXAAiADQANAAvADIAOABcACIALAAgADQANAAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB4AFwAIgAsACAAXAAiADQANgAvADEANABcACIALAAgADQANgAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwBcACIALAAgAFwAIgAyADgALwAxADIAXAAiACwAIAAyADgALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgAgAEwAaQBtAGUAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBNAFYATwBDAFwAIgAsACAAXAAiADEANAAvADEAMgBcACIALAAgADEANAAsACAAMQAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABOADIATwBcAG4ARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBXAFAATgAyAE8AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAYQBzAFwAIgAsACAAXAAiAEMATwAyAC0AZQAgAGYAYQBjAHQAbwByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAE8AMgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIAAyADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEYANABcACIALAAgADYANgAzADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwAyAEYANgBcACIALAAgADEAMgAyADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEYANgBcACIALAAgADIAMgA4ADAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEYAMwBcACIALAAgADEANwAyADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwB0AGEAdABlAHMAIABhAG4AZAAgAHQAZQByAHIAaQB0AG8AcgBpAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUALwBUAGUAcgByAGkAdABvAHIAeQBcACIALAAgAFwAIgBDAG8AbQBtAG8AbgAgAE4AYQBtAGUAXAAiACwAIABcACIAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AZQB3ACAAUwBvAHUAdABoACAAVwBhAGwAZQBzAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQwBhAHAAaQB0AGEAbAAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBpAGMAdABvAHIAaQBhAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBRAHUAZQBlAG4AcwBsAGEAbgBkAFwAIgAsACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAbwB1AHQAaAAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFMAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIALAAgAFwAIgBXAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAGEAcwBtAGEAbgBpAGEAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AbwByAHQAaABlAHIAbgAgAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAE4AVABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBCAFMAIABTAHQAYQB0AGkAcwB0AGMAYQBsACAAQQByAGUAYQBzACAATABlAHYAZQBsACAANAAgAC0AIABXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAEIAdQByAGUAYQB1ACAAbwBmACAAUwB0AGEAdABpAHMAdABpAGMAcwAgACgAQQBCAFMAKQAgAC0AIABTAHQAYQB0AGkAcwB0AGkAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAAyACAALQAgADIAMAAyADEAIAAtACAAUwBoAGEAcABlAGYAaQBsAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAQQAgADQAIABOAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAbgBiAHUAcgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAbgBkAHUAcgBhAGgAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABJAG4AbgBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABFAGEAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAATgBvAHIAdABoACAAVwBlAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABTAG8AdQB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAAVwBoAGUAYQB0ACAAQgBlAGwAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhACAALQAgAE8AdQB0AGIAYQBjAGsAIAAoAE4AbwByAHQAaAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgAUwBvAHUAdABoACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAyADoAIABUAHIAYQBuAHMAbABhAHQAaQBuAGcAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACAAdABvACAAdwBlAHQAIABhAG4AZAAgAGQAcgB5ACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAALQAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBGAHIAeQBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AEQAcgB5AFwAdQAwADAAMgA3AC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAbwByACAARAByAHkAIABaAG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAaABpAGcAaAAgAHQAZQBtAHAAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABpAG4AIABNAEEAVAAgAHYAYQBsAHUAZQAgAGYAbwByACAAdwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAYwBoAGEAbgBnAGUAZAAgADEAMAAgAHQAbwAgADEAMQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABtAGkAbgAgAGEAbgBkACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAZgBvAHIAIABNAEEAVAAsACAATQBBAFAALAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIALAAgAGUAbABlAHYAYQB0AGkAbwBuACwAIABNAEEAUAA6AFAARQBUACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlAHMAIABmAHIAbwBtACAAcgBlAGEAbAAgAGMAbABpAG0AYQB0AGUAIABkAGEAdABhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAQQBGACAAYQBjAGMAZQBwAHQAcwAgAHIAYQBpAG4AZgBhAGwAbAAgAGEAcwAgAGEAIABwAHIAbwB4AHkAIABmAG8AcgAgAHAAcgBlAGMAaQBwAGkAdABhAHQAaQBvAG4ALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAEEAVABcACIALAAgAFwAIgBNAEEAUABcACIALAAgAFwAIgBGAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByAFwAIgAsACAAXAAiAEUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AYQB4ACAAdABlAG0AcABcACIALAAgAFwAIgBNAGkAbgAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGEAeAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBhAHgAIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AaQBuACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBhAHgAIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AbgB0AGEAbgBlAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAAMQAwADAAMAAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAHcAZQB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAOAAgAEMAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAMAAwACAAbQBtACAALQAgAGQiIAAyADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAuADAAMAAxACwAIAAyADAAMAAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAFwAdQAwADAAMwBlACAANgAwADAAbQBtAFwAIgAsACAANgAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIAQQBuAG4AdQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkIiAANgAwADAAbQBtAFwAIgAsACAALQA5ADkAOQA5ADkAOQAsACAANgAwADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABaAG8AbgBlAFwAIgAsACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGMAcgBpAHQAZQByAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAbwBjAGMAdQByAHMAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAFwAdQAwADAAMwBlAKMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABlAGEAYwBoAGkAbgBnACAAZABvAGUAcwAgAG4AbwB0ACAAbwBjAGMAdQByAFwAIgAsACAAXAAiAKMDKAA12F/cNdhO3DXYVtw12FvcKQBkIqMDKAA12DjcNdhH3DAAKQArADXYYNw12FzcNdhW3DXYWdwgADXYZNw12E7cNdhh3DXYUtw12F/cIAAOITXYXNw12FncNdhR3DXYVtw12FvcNdhU3CAANdhQ3DXYTtw12F3cNdhO3DXYUNw12FbcNdhh3DXYZtxcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcwAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAXAAiAEYAcgBhAGMAVwBFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFkAZQBzACAALQAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAC0AIABuAG8AdAAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAGQAYQB0AGEAIABzAGMAbwByAGUAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABYAFgAWABYAFgAWABYAFgAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABhAHQAYQAgAHMAbwB1AHIAYwBlAFwAIgAsACAAXAAiAEQAYQB0AGEAIABzAGMAbwByAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAbgB0AGUAcgBuAGEAdABpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlACAAbwByACAAcgBlAGcAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABpAG4AdABlAG4AcwBpAHQAeQAgAGMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAYQBwAHAAcgBvAHYAZQBkACAAbQBlAHQAaABvAGQAXAAiACwAIAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAZQByAGkAZgBpAGUAZAAgAGMAcgBlAGQAZQBuAHQAaQBhAGwAIABtAGEAdABjAGgAaQBuAGcAIABJAFMATwAxADQAMAA2ADcAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIABcAHUAMAAwADIANwBBAHIAZQBhAHMAIABhAHIAZQAgAHMAdQBiAGoAZQBjAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIAAoAGkALgBlAC4ALAAgAGkAbgAgAHQAaABlACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQApACAAdwBoAGUAbgAuAC4ALgAgAHQAaABlACAAbABhAG4AZAAgAGkAcwAgAGkAcgByAGkAZwBhAHQAZQBkACAAKABlAHgAYwBlAHAAdAAgAGQAcgBpAHAAIABpAHIAcgBpAGcAYQB0AGkAbwBuACkALgBcAHUAMAAwADIANwBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyADoAIABFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBQAFIAUAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABvAHIAIABwAGEAZABkAG8AYwBrAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBQAFIAUABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAAyAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABDAGgAYQBuAGcAZQBkACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAdQAwADAAMgA3ACAAdABvACAAcwBpAG4AZwB1AGwAYQByACAAXAB1ADAAMAAyADcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcAHUAMAAwADIANwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjADEAIABtAG8AbgB0AGgAXAAiACwAIABcACIARABlAGUAcAAgAEwAaQB0AHQAZQByAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABNAGEAbgB1AHIAZQAgACgAdwBpAHQAaAAvAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAcAByAG8AYwBlAHMAcwBpAG4AZwAgAGkAbgB0AG8AIABwAGUAbABsAGUAdABpAHoAZQBkACAAZgBlAHIAdABpAGwAaQBzAGUAcgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAsACAAUgBhAG4AZwBlACAAYQBuAGQAIABQAGEAZABkAG8AYwBrACAAKABjACkAKABkACkAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIjEAMABcACIALAAgADAALgA2ADYALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADEALAAgADAALgA2ADgALAAgADAALgAxACwAIAAwAC4AMQAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMgAsACAAMAAuADcALAAgADAALgAxACwAIAAwAC4AMQAzACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMwAsACAAMAAuADcAMQAsACAAMAAuADEALAAgADAALgAxADQALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQA0ACwAIAAwAC4ANwAzACwAIAAwAC4AMQAsACAAMAAuADEANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA1ACwAIAAwAC4ANwA0ACwAIAAwAC4AMQAsACAAMAAuADEANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANgAsACAAMAAuADcANQAsACAAMAAuADEALAAgADAALgAxADgALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADcALAAgADAALgA3ADYALAAgADAALgAxACwAIAAwAC4AMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOAAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADIALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADkALAAgADAALgA3ADcALAAgADAALgAxACwAIAAwAC4AMgA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAwACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIANgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMQAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAyADkALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADIALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMwAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAzACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANAAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgAzADcALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADUALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADYALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4ANAA0ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIAAyADcALAAgADAALgA4ACwAIAAwAC4AMQAsACAAMAAuADQAOAAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiMgA4AFwAIgAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANQAsACAAMAAuADAAMQAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBcACIALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAG0AYQBuAHUAcgBlACAAdwBpAHQAaABvAHUAdAAgAGIAZQBkAGQAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIATQBBAFQAIAByAGEAdwBcACIAIABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgAHIAbwB3ACAAbwBmACAATgBJAFIAIABNAE0AQQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBQAG8AdQBsAHQAcgB5ACAAdwBpAHQAaAAgAGEAbgBkACAAdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBNAEEAVAAgAHIAYQB3AFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGwAbABvAHcAIABsAG8AbwBrAHUAcAAgAG8AZgAgAG4AdQBtAGIAZQByAHMALgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAbgBkACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAHIAZQB0AHUAcgBuAGUAZAAgAHQAbwAgAHQAaABlACAAcwBvAGkAbABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAE4AaQAgAFwAdQAwADAAMgA2ACAARQBGAE4AMgBPAGkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAxAC4ANABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAxADAALgAxADoAIABXAGEAcwB0AGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADEAMAAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AbABpAGQAIABXAGEAcwB0AGUAIABUAHIAZQBhAHQAbQBlAG4AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHcAYQBzAHQAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABiAHkAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAXABuAEUAXwBnAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBfAGcAPQBcAFwAcwB1AG0AXwB0AFwAXABzAHUAbQBfAHcAKABRAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB3AHQAZwApAFwAbgBRAF8AdwB0ACAAPQAgAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAG8AZgAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAsACAAbwBuACAAYQAgAHcAZQB0ACAAdwBlAGkAZwBoAHQAIABiAGEAcwBpAHMAIAAoAHQAKQBcAG4ARQBGAF8AdwB0AGcAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwAgAGcAIABmAG8AcgAgAHQAaABlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAHcAYQBzAHQAZQAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdAAgACgAdAAgAEMATwAyAGUALwB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABRAF8AdwB0ACwAIABFAEYAXwB3AHQAZwAsAFwAbgAgACAAIAAgAFEAXwB3AHQAIAAqACAARQBGAF8AdwB0AGcAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIAB3AGEAcwB0AGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAYgB5ACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AZwA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AdABcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAHcAKABRAF8AewB3AHQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewB3AHQAZwB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIABvAGYAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQALAAgAG8AbgAgAGEAIAB3AGUAdAAgAHcAZQBpAGcAaAB0ACAAYgBhAHMAaQBzAFwAIgAsACAAXAAiAHQAXAAiACwAIABcACIAUwB1AG0AIABvAGYAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAHcAdABnAFwAIgAsACAAXAAiAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABnAHIAZQBlAG4AaABvAHUAcwBlACAAZwBhAHMAIABnACAAZgBvAHIAIAB0AGgAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABvAGYAIAB3AGEAcwB0AGUAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAXAAiACwAIABcACIAdAAgAEMATwAyAGUALwB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGcAXAAiACwAIABcACIAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAHYAbwBsAHcAdABcACIALAAgAFwAIgBxAHUAYQBuAHQAaQB0AHkAIABvAGYAIABzAG8AbABkACAAdwBhAHMAdABlACAAaQBuAHAAdQB0ACAAYQBzACAAdgBvAGwAdQBtAGUAIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAdABvAG4AbgBlAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAxADAALgAxAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBfAG0AYQBzAHMAdwB0AFwAIgAsACAAXAAiAHEAdQBhAG4AdABpAHQAeQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AYQBzAHMAXAAiACwAIABcACIAdABvAG4AbgBlAHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABRAF8AdgBvAGwAdwB0ACAAYQBuAGQAIABRAF8AbQBhAHMAcwB3AHQAIAB2AGEAcgBpAGEAYgBsAGUAcwAgAHQAbwAgAGMAbABlAGEAcgBsAHkAIAB0AHIAYQBjAGsAIABpAG4AcAB1AHQAIABvAHIAIABjAGEAbABjAHUAbABhAHQAZQBkACAAUQAgAHYAYQBsAHUAZQBzAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXABuAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXABuAFEAXwB3AHQAXABuAHQAXABuAFEAXwB3AHQAPQBWAF8AdwB0AFwAXAB0AGkAbQBlAHMAIABWAFQATQBfAHcAXABuAFYAXwB3AHQAIAA9ACAAdgBvAGwAdQBtAGUAIABvAGYAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgAGIAZQBpAG4AZwAgAHMAZQBuAHQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQAgAHQAIAAoAG0AMwApAFwAbgBWAFQATQBfAHcAIAA9ACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwAgACgAdAAvAG0AMwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAXwB3AHQALAAgAFYAVABNAF8AdwAsAFwAbgAgACAAIAAgAFYAXwB3AHQAIAAqACAAVgBUAE0AXwB3AFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIAB3AGEAcwB0AGUAIABmAHIAbwBtACAAdwBhAHMAdABlACAAdgBvAGwAdQBtAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBRAF8AdwB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADEAMAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFEAXwB7AHcAdAB9AD0AVgBfAHsAdwB0AH0AXABcAHQAaQBtAGUAcwAgAFYAVABNAF8AdwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBfAHcAdABcACIALAAgAFwAIgB2AG8AbAB1AG0AZQAgAG8AZgAgAHMAbwBsAGkAZAAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAIAB3ACAAYgBlAGkAbgBnACAAcwBlAG4AdAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAZgBhAGMAaQBsAGkAdAB5ACAAdABcACIALAAgAFwAIgBtADMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFQATQBfAHcAXAAiACwAIABcACIAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAbwBmACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAZgBvAHIAIAB3AGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgB0AC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdwBcACIALAAgAFwAIgB3AGEAcwB0AGUAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAdABcACIALAAgAFwAIgB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAeQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAHcAYQBzAHQAZQBzACAAZABpAHMAcABvAHMAZQBkACAAbwBmACAAYQB0ACAAZABpAGYAZgBlAHIAZQBuAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGYAYQBjAGkAbABpAHQAaQBlAHMAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIARQBGAHcAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBVAG4AaQB0AFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAdAAgAEMATwAyAGUAIAAvACAAdABcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADEAXAAiACkAKQA7AFwAbgBcAG4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzADUALAAgADQALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIAB0AHkAcABlACAAdABcACIALAAgAFwAIgBXAGEAcwB0AGUAIAB0AHkAcABlACAAdwBcACIALAAgAFwAIgBFAEYAdwB0AFwAIgAsACAAXAAiAEUARgAgAHMAbwB1AHIAYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAyAC4AMQAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgADEALgA2ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4ANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAyAC4AMAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAdABhAGIAbABlACAAMQA1AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEwAYQBuAGQAZgBpAGwAbABcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgADAALgA0ACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMwAuADMALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIASQBuAGUAcgB0ACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAbwBuAGMAcgBlAHQAZQAsACAAbQBlAHQAYQBsACwAIABwAGwAYQBzAHQAaQBjACAAbwByACAAZwBsAGEAcwBzACkAXAAiACwAIAAwACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMQAuADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAbgBkAGYAaQBsAGwAXAAiACwAIABcACIAQwBvAG0AbQBlAHIAYwBpAGEAbAAgAGEAbgBkACAAaQBuAGQAdQBzAHQAcgBpAGEAbAAgAHcAYQBzAHQAZQBcACIALAAgADEALgAzACwAIABcACIATgBHAEEARgAgADIAMAAyADUAIAB0AGEAYgBsAGUAIAAxADUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIATABhAG4AZABmAGkAbABsAFwAIgAsACAAXAAiAEMAbwBuAHMAdAByAHUAYwB0AGkAbwBuACAAYQBuAGQAIABkAGUAbQBvAGwAaQB0AGkAbwBuACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADIALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAHQAYQBiAGwAZQAgADEANQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUALAAgAGcAcgBlAGUAbgAgAHcAYQBzAHQAZQAsACAAdwBvAG8AZAAsACAAcwBsAHUAZABnAGUAXAAiACwAIAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAVwBvAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAMAAuADAAMQA2ADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBUAGUAeAB0AGkAbABlAHMAXAAiACwAIAAwAC4AMwA2ADYANwAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADQAOQAxADkALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AZQByAHQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwBvAG4AYwByAGUAdABlACwAIABtAGUAdABhAGwALAAgAHAAbABhAHMAdABpAGMAIABvAHIAIABnAGwAYQBzAHMAKQBcACIALAAgADAALgAxADEAMAAwACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIASQBuAGMAaQBuAGUAcgBhAHQAaQBvAG4AXAAiACwAIABcACIATQB1AG4AaQBjAGkAcABhAGwAIABzAG8AbABpAGQAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA1ADMANwAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBjAGkAbgBlAHIAYQB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAxAC4ANgA0ADkALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOABcACIAOwBcAG4AXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMAA0ADYALAAgAFwAIgBOAEcAQQBGACAAMgAwADIANQAgAFQAYQBiAGwAZQAgADEAOQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEYAbwBvAGQAIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYQBuAGkAbQBhAGwAIABjAGEAcgBjAGEAcwBzAGUAcwAsACAAcwBwAG8AaQBsAGUAZAAgAGEAbgBpAG0AYQBsACAAZgBlAGUAZAAgAG8AcgAgAGMAcgBvAHAAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnAFwAIgAsACAAXAAiAEcAcgBlAGUAbgAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAbwByACAAcAByAHUAbgBpAG4AZwBzACkAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBXAG8AbwBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAXAAiACwAIABcACIAUwBsAHUAZABnAGUAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwBcACIALAAgAFwAIgBQAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAEEAbABsACAAbwByAGcAYQBuAGkAYwAgAHcAYQBzAHQAZQBcACIALAAgADAALgAwADIAOAAsACAAXAAiAE4ARwBBAEYAIAAyADAAMgA1ACAAVABhAGIAbABlACAAMQA5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARgBvAG8AZAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABhAG4AaQBtAGEAbAAgAGMAYQByAGMAYQBzAHMAZQBzACwAIABzAHAAbwBpAGwAZQBkACAAYQBuAGkAbQBhAGwAIABmAGUAZQBkACAAbwByACAAYwByAG8AcAApAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAaQBvAG4AXAAiACwAIABcACIARwByAGUAZQBuACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGMAcgBvAHAAIAByAGUAcwBpAGQAdQBlAHMAIABvAHIAIABwAHIAdQBuAGkAbgBnAHMAKQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFcAbwBvAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgBcACIALAAgAFwAIgBTAGwAdQBkAGcAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGQAaQBnAGUAcwB0AGkAbwBuAFwAIgAsACAAXAAiAFAAYQBwAGUAcgAgAGEAbgBkACAAYwBhAHIAZABiAG8AYQByAGQAXAAiACwAIABcACIAXAAiACwAIABcACIAXAAiAFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAcwBGAG8AcgBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAAxACwAXABuACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAXAB1ADAAMAAyADcAcABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBiAG8AYQByAGQAXAB1ADAAMAAyADcAIAB0AG8AIABcAHUAMAAwADIANwBwAGEAcABlAHIAIABhAG4AZAAgAGMAYQByAGQAYgBvAGEAcgBkAFwAdQAwADAAMgA3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIABcAHUAMAAwADIANwBwAHIAdQBuAG4AaQBuAGcAcwBcAHUAMAAwADIANwAgAHQAbwAgAFwAdQAwADAAMgA3AHAAcgB1AG4AaQBuAGcAcwBcAHUAMAAwADIANwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABFAEYAIABzAG8AdQByAGMAZQAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAHMAcABlAGMAaQBmAGkAYwAgAHIAZQBmAGUAcgBlAG4AYwBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBJAG4AYwBpAG4AZQByAGEAdABpAG8AbgA6ACAARgBvAG8AZAAgAHcAYQBzAHQAZQAsACAAZwByAGUAZQBuACAAdwBhAHMAdABlACwAIAB3AG8AbwBkACwAIABzAGwAdQBkAGcAZQBcAHUAMAAwADIANwAgAGkAbgAgAG8AcgBkAGUAcgAgAHQAbwAgAHUAcwBlACAAdgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAdgBhAGwAdQBlAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAcwB1AGIALQBjAGEAdABlAGcAbwByAGkAZQBzACAAZgBvAHIAIABcAHUAMAAwADIANwBDAG8AbQBwAG8AcwB0AGkAbgBnADoAIABBAGwAbAAgAG8AcgBnAGEAbgBpAGMAIAB3AGEAcwB0AGUAXAB1ADAAMAAyADcAIABpAG4AIABvAHIAZABlAHIAIAB0AG8AIAB1AHMAZQAgAHYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHYAYQBsAHUAZQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHMAdQBiAC0AYwBhAHQAZQBnAG8AcgBpAGUAcwAgAGYAbwByACAAXAB1ADAAMAAyADcAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABpAG8AbgA6ACAAQQBsAGwAIABvAHIAZwBhAG4AaQBjACAAdwBhAHMAdABlAFwAdQAwADAAMgA3ACAAaQBuACAAbwByAGQAZQByACAAdABvACAAdQBzAGUAIAB2AG8AbAB1AG0AZQAgAHQAbwAgAG0AYQBzAHMAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIAB2AGEAbAB1AGUAcwBcACIAXABuACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AKQApACkAOwBcAG4AXABuAFwAbgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFQAYQBiAGwAZQAgAEEALgA0AC4AMQAuADIAOgAgAFYAbwBsAHUAbQBlACAAdABvACAAbQBhAHMAcwAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdgBhAHIAaQBvAHUAcwAgAHcAYQBzAHQAZQAgAHQAeQBwAGUAcwAgACgAdAAvAG0AMwApACAAKABWAFQATQB3ACkAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVABpAHQAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBvAGwAdQBtAGUAIAB0AG8AIABtAGEAcwBzACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB2AGEAcgBpAG8AdQBzACAAdwBhAHMAdABlACAAdAB5AHAAZQBzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBUAE0AdwBcACIAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFUAbgBpAHQAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgB0AC8AbQAzAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4ANAAuADEALgAyAFwAIgApACkAOwBcAG4AXABuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8ARABhAHQAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADIALAAgADIALABcAG4AIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIABcACIAVwBhAHMAdABlACAAdAB5AHAAZQAgAHcAXAAiACwAIABcACIAVgBUAE0AdwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AbwBkACAAdwBhAHMAdABlACAAKABpAG4AYwBsAHUAZABpAG4AZwAgAGEAbgBpAG0AYQBsACAAYwBhAHIAYwBhAHMAcwBlAHMALAAgAHMAcABvAGkAbABlAGQAIABhAG4AaQBtAGEAbAAgAGYAZQBlAGQAIABvAHIAIABjAHIAbwBwACkAXAAiACwAIAAwAC4ANQAwADsAXABuACAAIAAgACAAIAAgACAAIABcACIAUABhAHAAZQByACAAYQBuAGQAIABjAGEAcgBkAGIAbwBhAHIAZABcACIALAAgADAALgAwADkAOwBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBHAHIAZQBlAG4AIAB3AGEAcwB0AGUAIAAoAGkAbgBjAGwAdQBkAGkAbgBnACAAYwByAG8AcAAgAHIAZQBzAGkAZAB1AGUAcwAgAG8AcgAgAHAAcgB1AG4AaQBuAGcAcwApAFwAIgAsACAAMAAuADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFcAbwBvAGQAXAAiACwAIAAwAC4AMQA1ADsAXABuACAAIAAgACAAIAAgACAAIABcACIAVABlAHgAdABpAGwAZQBzAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFMAbAB1AGQAZwBlAFwAIgAsACAAMAAuADcAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFIAdQBiAGIAZQByACAAYQBuAGQAIABsAGUAYQB0AGgAZQByAFwAIgAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEkAbgBlAHIAdAAgAHcAYQBzAHQAZQAgACgAaQBuAGMAbAB1AGQAaQBuAGcAIABjAG8AbgBjAHIAZQB0AGUALAAgAG0AZQB0AGEAbAAsACAAcABsAGEAcwB0AGkAYwAgAG8AcgAgAGcAbABhAHMAcwApAFwAIgAsACAAMAAuADQAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBuAGkAYwBpAHAAYQBsACAAcwBvAGwAaQBkACAAdwBhAHMAdABlAFwAIgAsACAAMAAuADMANgA7AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBtAG0AZQByAGMAaQBhAGwAIABhAG4AZAAgAGkAbgBkAHUAcwB0AHIAaQBhAGwAIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwAzADsAXABuACAAIAAgACAAIAAgACAAIABcACIAQwBvAG4AcwB0AHIAdQBjAHQAaQBvAG4AIABhAG4AZAAgAGQAZQBtAG8AbABpAHQAaQBvAG4AIAB3AGEAcwB0AGUAXAAiACwAIAAwAC4AMwA5AFwAbgAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACkAKQApADsAXABuAFwAbgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBoAGEAbgBnAGUAZAAgAGMAbwBsAHUAbQBuACAAaABlAGEAZABlAHIAIABDAEYAdwAgAHQAbwAgAFYAVABNAHcAIAB0AG8AIABtAGEAdABjAGgAIAB0AGkAdABsAGUAIAB2AGEAcgBpAGEAYgBsAGUALgBcACIAKQApADsAXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAXwBTAHUAbQBXAGEAcwB0AGUAVAByAGUAYQB0AG0AZQBuAHQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVwBhAHMAdABlAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVQBuAGkAdABBAHIAcgBhAHkALAAgAEEAbQBvAHUAbgB0AEEAcgByAGEAeQAsAFwAbgAgACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsACAAVwBhAHMAdABlAFQAeQBwAGUALAAgAFQAcgBlAGEAdABtAGUAbgB0AEwAbwBjAGEAdABpAG8AbgBUAHkAcABlACwAIABVAG4AaQB0AFQAeQBwAGUALABcAG4AIAAgAFMAVQBNAEkARgBTACgAXABuACAAIAAgACAAQQBtAG8AdQBuAHQAQQByAHIAYQB5ACwAXABuACAAIAAgAFQAcgBlAGEAdABtAGUAbgB0AEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQAVAB5AHAAZQAsAFwAbgAgACAAIAAgAFcAYQBzAHQAZQBBAHIAcgBhAHkALAAgAFcAYQBzAHQAZQBUAHkAcABlACwAXABuACAAIAAgACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAVAByAGUAYQB0AG0AZQBuAHQATABvAGMAYQB0AGkAbwBuAFQAeQBwAGUALAAgAFwAbgAgACAAIAAgAFUAbgBpAHQAQQByAHIAYQB5ACwAIABVAG4AaQB0AFQAeQBwAGUAXABuACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADEAXwBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFcAYQBzAHQAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAxAF8ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBXAGEAcwB0AGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMQBfAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AVwBhAHMAdABlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFQAaQB0AGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAFUAbgBpAHQAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMQAwAF8AMQBfADEAXwAxAF8AXwAyAF8ATQBhAHMAcwBPAGYAVwBhAHMAdABlAEYAcgBvAG0AVgBvAGwAdQBtAGUAXwBTAG8AdQByAGMAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADEAMABfADEAXwAxAF8AMQBfAF8AMgBfAE0AYQBzAHMATwBmAFcAYQBzAHQAZQBGAHIAbwBtAFYAbwBsAHUAbQBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAxADAAXwAxAF8AMQBfADEAXwBfADIAXwBNAGEAcwBzAE8AZgBXAGEAcwB0AGUARgByAG8AbQBWAG8AbAB1AG0AZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVABpAHQAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFMAbwB1AHIAYwBlACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAHMARgBvAHIAVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0AF8ARABhAHQAYQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBzAEYAbwByAFcAYQBzAHQAZQBUAHIAZQBhAHQAbQBlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AVwBhAHMAdABlAF8AVwBhAHMAdABlAFYAbwBsAHUAbQBlAFQAbwBNAGEAcwBzAEMAbwBuAHYAZQByAHMAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AVQBuAGkAdAAiACwAIgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFcAYQBzAHQAZQBfAFcAYQBzAHQAZQBWAG8AbAB1AG0AZQBUAG8ATQBhAHMAcwBDAG8AbgB2AGUAcgBzAGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAEQAYQB0AGEAIgAsACIAVwBhAHMAdABlAFMAbwBsAGkAZABfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBXAGEAcwB0AGUAXwBXAGEAcwB0AGUAVgBvAGwAdQBtAGUAVABvAE0AYQBzAHMAQwBvAG4AdgBlAHIAcwBpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFcAYQBzAHQAZQBTAG8AbABpAGQAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBXAGEAcwB0AGUAUwBvAGwAaQBkAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAF8AUwB1AG0AVwBhAHMAdABlAFQAcgBlAGEAdABtAGUAbgB0ACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16612,10 +16620,29 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>